<commit_message>
Clear the Release sweep contradiction on the Roadmap
The Roadmap still carried a "Daily sweep releasing titles from
long-inactive holders" task and a ledger tracking last-seen timestamps.
Both predate the DECIDED row on the decision sheet - titles are held
forever, nothing is ever released, and the ledger is append-only.

Deleting the sweep outright would have left a real gap: Contested is
the one revocable scarcity type and Phase 4 had no row for the takeover
path. Replaced rather than removed.

- Server ledger: append-only, tracks Limited/Founding/Unique/Contested
  claims, no last-seen timestamps
- Release sweep -> Contested transfer: score-beats-holder takeover,
  never on death and never on inactivity

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/TitlesMod-Design.xlsx
+++ b/design/TitlesMod-Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\IdeaProjects\TitlesMod\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3BA2105B-EB3E-49C3-B00E-431FBF682AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{852F5E69-9E51-4409-B7A7-6753D8C09D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5112" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{CA22B986-27D2-4854-9A3A-FA10050CCE84}"/>
+    <workbookView xWindow="5112" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{2B6B08A0-D99A-4FBE-A4B8-D7F51C61483B}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -4644,7 +4644,7 @@
     <t>Server ledger</t>
   </si>
   <si>
-    <t>SavedData tracking Limited and Unique claims plus last-seen timestamps</t>
+    <t>Append-only SavedData tracking Limited - Founding - Unique and Contested claims. No last-seen timestamps - nothing is ever released so they are never read</t>
   </si>
   <si>
     <t>Ledger persists across restarts</t>
@@ -4659,13 +4659,13 @@
     <t>No double-grants under race</t>
   </si>
   <si>
-    <t>Release sweep</t>
-  </si>
-  <si>
-    <t>Daily sweep releasing titles from long-inactive holders</t>
-  </si>
-  <si>
-    <t>Latecomers can chase Limited titles</t>
+    <t>Contested transfer</t>
+  </si>
+  <si>
+    <t>Score-beats-holder takeover for Contested titles - the only revocable scarcity type. Never on death and never on inactivity</t>
+  </si>
+  <si>
+    <t>The Unrivaled changes hands only when someone beats the score</t>
   </si>
   <si>
     <t>Ledger UI</t>
@@ -6289,7 +6289,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A36E9414-1507-41FE-B199-442930F37D0F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0695F88D-2251-4452-ADB7-A833A1F80A7F}">
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6572,13 +6572,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1" xr:uid="{A36E9414-1507-41FE-B199-442930F37D0F}"/>
+  <autoFilter ref="A1:C1" xr:uid="{0695F88D-2251-4452-ADB7-A833A1F80A7F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{258A1ABF-5747-4C43-B595-EDB8A92217E7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F1EEEC-C9A8-4474-98CA-AB18E193254C}">
   <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7176,13 +7176,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{258A1ABF-5747-4C43-B595-EDB8A92217E7}"/>
+  <autoFilter ref="A1:D1" xr:uid="{56F1EEEC-C9A8-4474-98CA-AB18E193254C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D736BB-E499-4EDC-9E1F-CFE025B6BF31}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C992350-FB65-4B54-9DDD-87E7A3F8BB41}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7240,13 +7240,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{E1D736BB-E499-4EDC-9E1F-CFE025B6BF31}"/>
+  <autoFilter ref="A1:G1" xr:uid="{0C992350-FB65-4B54-9DDD-87E7A3F8BB41}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{481FF3C1-0E29-460C-A44C-F53E065B77E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A60416-8C94-4039-B79F-9FC745818C7C}">
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7904,13 +7904,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{481FF3C1-0E29-460C-A44C-F53E065B77E4}"/>
+  <autoFilter ref="A1:G1" xr:uid="{30A60416-8C94-4039-B79F-9FC745818C7C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48CCB69A-E489-4474-8A32-E59654D5B332}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FB977C9-040A-4C95-BE5D-44270507B9D8}">
   <dimension ref="A1:Q104"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -13442,13 +13442,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1" xr:uid="{48CCB69A-E489-4474-8A32-E59654D5B332}"/>
+  <autoFilter ref="A1:Q1" xr:uid="{8FB977C9-040A-4C95-BE5D-44270507B9D8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFE02F57-E7DC-416C-8FC9-E22D39861831}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85C5910A-D221-4564-B410-2A9DA9866023}">
   <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -14139,13 +14139,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{AFE02F57-E7DC-416C-8FC9-E22D39861831}"/>
+  <autoFilter ref="A1:H1" xr:uid="{85C5910A-D221-4564-B410-2A9DA9866023}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E92F506-C0AD-4FDD-8814-AB63D37ED662}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{357492CC-8CCD-4773-BB2A-C85A610D7D53}">
   <dimension ref="A1:H46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -15353,13 +15353,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{0E92F506-C0AD-4FDD-8814-AB63D37ED662}"/>
+  <autoFilter ref="A1:H1" xr:uid="{357492CC-8CCD-4773-BB2A-C85A610D7D53}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A44C572-131D-44C1-8CEA-FA86469E3B4E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00877D96-D750-4FC6-B5F4-99811411F11A}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -15839,13 +15839,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{2A44C572-131D-44C1-8CEA-FA86469E3B4E}"/>
+  <autoFilter ref="A1:H1" xr:uid="{00877D96-D750-4FC6-B5F4-99811411F11A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8513E5B-B681-4E6A-8167-A344986C3D21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD22849-313C-4951-A781-8DF4AE51A0C2}">
   <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16230,13 +16230,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{E8513E5B-B681-4E6A-8167-A344986C3D21}"/>
+  <autoFilter ref="A1:E1" xr:uid="{9FD22849-313C-4951-A781-8DF4AE51A0C2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184E8F60-124B-41FC-9457-DC42B2E004EB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2069EE06-F3A2-4A71-9ADB-E58B981251AE}">
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16962,13 +16962,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{184E8F60-124B-41FC-9457-DC42B2E004EB}"/>
+  <autoFilter ref="A1:G1" xr:uid="{2069EE06-F3A2-4A71-9ADB-E58B981251AE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE481AD0-D06D-45B6-942A-385A9594135C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D719F90B-D691-4214-B12A-E5DD09CE79F0}">
   <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -17549,7 +17549,7 @@
         <v>1455</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>1524</v>
       </c>
@@ -17601,7 +17601,7 @@
         <v>1455</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>1524</v>
       </c>
@@ -18252,13 +18252,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{CE481AD0-D06D-45B6-942A-385A9594135C}"/>
+  <autoFilter ref="A1:H1" xr:uid="{D719F90B-D691-4214-B12A-E5DD09CE79F0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F9B2B16-048D-4ED1-B895-B90C6006F60D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCEA78DE-E434-4753-AF33-C69E10F5DC44}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18609,7 +18609,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{6F9B2B16-048D-4ED1-B895-B90C6006F60D}"/>
+  <autoFilter ref="A1:E1" xr:uid="{BCEA78DE-E434-4753-AF33-C69E10F5DC44}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>